<commit_message>
Deepen metro reference: TV affiliates, radio groups, agencies + Quick-Start tab
- metro_reference.py: METRO_BROADCAST dict for all 42 metros - Big-4 TV
  affiliate call signs, major radio ownership groups (Audacy/iHeart/Bonneville/
  Hubbard/Cox etc. with flagship stations), and notable ad agencies per market
  (W+K Portland, Martin Agency Richmond, GSD&M Austin, R&R Vegas, VML KC...).
- US Metro Reference sheet widened to 13 columns with TV/Radio/Agencies.
- New Quick-Start by Metro tab: per market - OOH rate band, top local OOH
  operators (auto-selected from scraped dataset: local/regional first, by
  confidence), TV, radio, newspaper, agencies to call, plus a universal
  foundation note (GBP+LSA+reviews -> SEO city pages -> geofenced paid ->
  local media).
- Legend + README updated; broadcast/agency data marked reference-level.
- Workbook now 31 sheets.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0169X7FqU7js4G1ZKY5WjVsV
</commit_message>
<xml_diff>
--- a/marketing-repository/data/BSymbolic_Marketing_Master_Expanded.xlsx
+++ b/marketing-repository/data/BSymbolic_Marketing_Master_Expanded.xlsx
@@ -36,7 +36,8 @@
     <sheet name="Cause and Community" sheetId="27" state="visible" r:id="rId27"/>
     <sheet name="US Metro Reference" sheetId="28" state="visible" r:id="rId28"/>
     <sheet name="Metro OOH Companies" sheetId="29" state="visible" r:id="rId29"/>
-    <sheet name="PBC Priority Playbook" sheetId="30" state="visible" r:id="rId30"/>
+    <sheet name="Quick-Start by Metro" sheetId="30" state="visible" r:id="rId30"/>
+    <sheet name="PBC Priority Playbook" sheetId="31" state="visible" r:id="rId31"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Master List'!$A$2:$G$1118</definedName>
@@ -65,8 +66,9 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="24" hidden="1">'Branding and Creative'!$A$2:$F$22</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="25" hidden="1">'B2B and Account-Based'!$A$2:$F$22</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="26" hidden="1">'Cause and Community'!$A$2:$F$17</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="27" hidden="1">'US Metro Reference'!$A$2:$J$44</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="27" hidden="1">'US Metro Reference'!$A$2:$M$44</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="28" hidden="1">'Metro OOH Companies'!$A$2:$H$112</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="29" hidden="1">'Quick-Start by Metro'!$A$2:$I$44</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -75,7 +77,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -94,6 +96,10 @@
     <font>
       <b val="1"/>
       <color rgb="FFFFFFFF"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <i val="1"/>
     </font>
   </fonts>
   <fills count="7">
@@ -155,7 +161,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -182,6 +188,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -671,7 +680,7 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>US Metro Reference = 42 largest markets with DMA rank, population, OOH rate band, # billboard operators, dominant newspaper &amp; business journal. Metro OOH Companies = 110 scraped billboard/OOH operators by metro. Turns the tactic menu into a US market reference.</t>
+          <t>US Metro Reference = 42 largest markets with DMA rank, population, OOH rate band, # billboard operators, newspaper, business journal, Big-4 TV affiliates, major radio groups &amp; notable ad agencies. Metro OOH Companies = 110 scraped billboard/OOH operators by metro. Quick-Start by Metro = who to call in each market (top local OOH operators, TV/radio/paper, agencies) + the universal foundation steps. TV/radio/agency data is reference-level - verify before buying.</t>
         </is>
       </c>
     </row>
@@ -53836,7 +53845,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J44"/>
+  <dimension ref="A1:M44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -53846,9 +53855,12 @@
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="15" customWidth="1" min="6" max="6"/>
     <col width="9" customWidth="1" min="7" max="7"/>
-    <col width="30" customWidth="1" min="8" max="8"/>
-    <col width="30" customWidth="1" min="9" max="9"/>
-    <col width="55" customWidth="1" min="10" max="10"/>
+    <col width="28" customWidth="1" min="8" max="8"/>
+    <col width="26" customWidth="1" min="9" max="9"/>
+    <col width="34" customWidth="1" min="10" max="10"/>
+    <col width="36" customWidth="1" min="11" max="11"/>
+    <col width="34" customWidth="1" min="12" max="12"/>
+    <col width="48" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -53866,6 +53878,9 @@
       <c r="H1" s="2" t="n"/>
       <c r="I1" s="2" t="n"/>
       <c r="J1" s="2" t="n"/>
+      <c r="K1" s="2" t="n"/>
+      <c r="L1" s="2" t="n"/>
+      <c r="M1" s="2" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
@@ -53914,6 +53929,21 @@
         </is>
       </c>
       <c r="J2" s="5" t="inlineStr">
+        <is>
+          <t>Big-4 TV Affiliates</t>
+        </is>
+      </c>
+      <c r="K2" s="5" t="inlineStr">
+        <is>
+          <t>Major Radio Groups</t>
+        </is>
+      </c>
+      <c r="L2" s="5" t="inlineStr">
+        <is>
+          <t>Notable Ad Agencies</t>
+        </is>
+      </c>
+      <c r="M2" s="5" t="inlineStr">
         <is>
           <t>Market Notes</t>
         </is>
@@ -53961,6 +53991,21 @@
       </c>
       <c r="J3" s="7" t="inlineStr">
         <is>
+          <t>WABC 7 · WCBS 2 · WNBC 4 · WNYW Fox 5</t>
+        </is>
+      </c>
+      <c r="K3" s="7" t="inlineStr">
+        <is>
+          <t>Audacy (WFAN, 1010 WINS) · iHeart (Z100) · SBS (Spanish, HQ)</t>
+        </is>
+      </c>
+      <c r="L3" s="7" t="inlineStr">
+        <is>
+          <t>Ogilvy, BBDO, Droga5, McCann (global HQs)</t>
+        </is>
+      </c>
+      <c r="M3" s="7" t="inlineStr">
+        <is>
           <t>Times Square spectaculars $10,000 to $1,000,000+/mo; Manhattan digital $15k–$50k; outer-borough static $3k–$8k.</t>
         </is>
       </c>
@@ -54007,6 +54052,21 @@
       </c>
       <c r="J4" s="7" t="inlineStr">
         <is>
+          <t>KABC 7 · KCBS 2 · KNBC 4 · KTTV Fox 11</t>
+        </is>
+      </c>
+      <c r="K4" s="7" t="inlineStr">
+        <is>
+          <t>iHeart (KIIS, KFI) · Audacy (KROQ, KNX) · Univision/SBS (Spanish)</t>
+        </is>
+      </c>
+      <c r="L4" s="7" t="inlineStr">
+        <is>
+          <t>Deutsch LA, 72andSunny, TBWA\Chiat\Day</t>
+        </is>
+      </c>
+      <c r="M4" s="7" t="inlineStr">
+        <is>
           <t>Iconic Sunset Strip bulletins command a large multiple of comparable units 30 mi east.</t>
         </is>
       </c>
@@ -54053,6 +54113,21 @@
       </c>
       <c r="J5" s="7" t="inlineStr">
         <is>
+          <t>WLS 7 · WBBM 2 · WMAQ 5 · WFLD Fox 32</t>
+        </is>
+      </c>
+      <c r="K5" s="7" t="inlineStr">
+        <is>
+          <t>Audacy (WBBM, WSCR) · iHeart · Nexstar (WGN Radio)</t>
+        </is>
+      </c>
+      <c r="L5" s="7" t="inlineStr">
+        <is>
+          <t>Leo Burnett, FCB Chicago, Energy BBDO</t>
+        </is>
+      </c>
+      <c r="M5" s="7" t="inlineStr">
+        <is>
           <t>Premium expressway (Kennedy/Dan Ryan) and Loop digital displays at the high end.</t>
         </is>
       </c>
@@ -54099,6 +54174,21 @@
       </c>
       <c r="J6" s="7" t="inlineStr">
         <is>
+          <t>KGO 7 · KPIX 5 · KNTV 11 · KTVU Fox 2</t>
+        </is>
+      </c>
+      <c r="K6" s="7" t="inlineStr">
+        <is>
+          <t>Audacy (KCBS) · iHeart · Bonneville</t>
+        </is>
+      </c>
+      <c r="L6" s="7" t="inlineStr">
+        <is>
+          <t>Goodby Silverstein, Duncan Channon, Argonaut</t>
+        </is>
+      </c>
+      <c r="M6" s="7" t="inlineStr">
+        <is>
           <t>Bay Area (SF/Oakland/San Jose); tech-driven demand and scarce inventory keep rates high.</t>
         </is>
       </c>
@@ -54145,6 +54235,21 @@
       </c>
       <c r="J7" s="7" t="inlineStr">
         <is>
+          <t>WSB 2 · WANF 46 · WXIA 11 · WAGA Fox 5</t>
+        </is>
+      </c>
+      <c r="K7" s="7" t="inlineStr">
+        <is>
+          <t>Cox Media Group (HQ, WSB) · iHeart · Urban One</t>
+        </is>
+      </c>
+      <c r="L7" s="7" t="inlineStr">
+        <is>
+          <t>22squared, Dagger, Chemistry</t>
+        </is>
+      </c>
+      <c r="M7" s="7" t="inlineStr">
+        <is>
           <t>Connector/I-285 'Perimeter' corridors; large billboard-friendly metro.</t>
         </is>
       </c>
@@ -54191,6 +54296,21 @@
       </c>
       <c r="J8" s="7" t="inlineStr">
         <is>
+          <t>WJLA 7 · WUSA 9 · WRC 4 · WTTG Fox 5</t>
+        </is>
+      </c>
+      <c r="K8" s="7" t="inlineStr">
+        <is>
+          <t>Hubbard (WTOP — top-billing US station) · iHeart · Cumulus (WMAL)</t>
+        </is>
+      </c>
+      <c r="L8" s="7" t="inlineStr">
+        <is>
+          <t>GMMB (political), RP3 Agency</t>
+        </is>
+      </c>
+      <c r="M8" s="7" t="inlineStr">
+        <is>
           <t>Billboards tightly limited in DC proper; value concentrated on MD/VA approaches &amp; transit.</t>
         </is>
       </c>
@@ -54237,6 +54357,21 @@
       </c>
       <c r="J9" s="7" t="inlineStr">
         <is>
+          <t>WCVB 5 · WBZ 4 · WBTS 10 · WFXT Fox 25</t>
+        </is>
+      </c>
+      <c r="K9" s="7" t="inlineStr">
+        <is>
+          <t>iHeart (WBZ-AM) · Audacy (WEEI) · Beasley</t>
+        </is>
+      </c>
+      <c r="L9" s="7" t="inlineStr">
+        <is>
+          <t>Hill Holliday, Arnold, MullenLowe, Allen &amp; Gerritsen</t>
+        </is>
+      </c>
+      <c r="M9" s="7" t="inlineStr">
+        <is>
           <t>OUTFRONT #1 with 675+ digital faces; I-93/Mass Pike and tunnel approaches priced highest.</t>
         </is>
       </c>
@@ -54283,6 +54418,21 @@
       </c>
       <c r="J10" s="7" t="inlineStr">
         <is>
+          <t>WFAA 8 · KTVT 11 · KXAS 5 · KDFW Fox 4</t>
+        </is>
+      </c>
+      <c r="K10" s="7" t="inlineStr">
+        <is>
+          <t>iHeart · Audacy (KRLD) · Cumulus (WBAP)</t>
+        </is>
+      </c>
+      <c r="L10" s="7" t="inlineStr">
+        <is>
+          <t>TRG (The Richards Group), Dieste (Hispanic)</t>
+        </is>
+      </c>
+      <c r="M10" s="7" t="inlineStr">
+        <is>
           <t>High-traffic corridors (I-35, LBJ, Central Expwy) priced highest.</t>
         </is>
       </c>
@@ -54329,6 +54479,21 @@
       </c>
       <c r="J11" s="7" t="inlineStr">
         <is>
+          <t>KTRK 13 · KHOU 11 · KPRC 2 · KRIV Fox 26</t>
+        </is>
+      </c>
+      <c r="K11" s="7" t="inlineStr">
+        <is>
+          <t>iHeart (KTRH) · Audacy · Cox (KKBQ)</t>
+        </is>
+      </c>
+      <c r="L11" s="7" t="inlineStr">
+        <is>
+          <t>Lopez Negrete (Hispanic), MMI Agency</t>
+        </is>
+      </c>
+      <c r="M11" s="7" t="inlineStr">
+        <is>
           <t>Clear Channel alone runs 2,000+ boards across 13 counties (99% of DMA adults).</t>
         </is>
       </c>
@@ -54375,6 +54540,21 @@
       </c>
       <c r="J12" s="7" t="inlineStr">
         <is>
+          <t>WPLG 10 · WFOR 4 · WTVJ 6 · WSVN Fox 7</t>
+        </is>
+      </c>
+      <c r="K12" s="7" t="inlineStr">
+        <is>
+          <t>iHeart · Cox · SBS (Spanish broadcasting HQ)</t>
+        </is>
+      </c>
+      <c r="L12" s="7" t="inlineStr">
+        <is>
+          <t>Zimmerman, Crispin (legacy), República Havas (Hispanic)</t>
+        </is>
+      </c>
+      <c r="M12" s="7" t="inlineStr">
+        <is>
           <t>I-95 / Palmetto / Dolphin Expwy and beach/tourism corridors carry premiums.</t>
         </is>
       </c>
@@ -54421,6 +54601,21 @@
       </c>
       <c r="J13" s="7" t="inlineStr">
         <is>
+          <t>WPVI 6 · KYW 3 · WCAU 10 · WTXF Fox 29</t>
+        </is>
+      </c>
+      <c r="K13" s="7" t="inlineStr">
+        <is>
+          <t>Audacy (HQ — KYW, WIP) · iHeart · Beasley (WMMR)</t>
+        </is>
+      </c>
+      <c r="L13" s="7" t="inlineStr">
+        <is>
+          <t>Digitas Philly (legacy), Brownstein Group, LevLane</t>
+        </is>
+      </c>
+      <c r="M13" s="7" t="inlineStr">
+        <is>
           <t>I-95 / Schuylkill Expwy and Center City digital at the top of range.</t>
         </is>
       </c>
@@ -54467,6 +54662,21 @@
       </c>
       <c r="J14" s="7" t="inlineStr">
         <is>
+          <t>WXYZ 7 · WWJ 62 · WDIV 4 · WJBK Fox 2</t>
+        </is>
+      </c>
+      <c r="K14" s="7" t="inlineStr">
+        <is>
+          <t>Audacy (WWJ, WXYT) · iHeart · Cumulus (WJR)</t>
+        </is>
+      </c>
+      <c r="L14" s="7" t="inlineStr">
+        <is>
+          <t>Doner, Campbell Ewald, Lafayette American</t>
+        </is>
+      </c>
+      <c r="M14" s="7" t="inlineStr">
+        <is>
           <t>I-75 / I-94 / M-10 corridors; International Outdoor runs 100+ Metro Detroit faces.</t>
         </is>
       </c>
@@ -54513,6 +54723,21 @@
       </c>
       <c r="J15" s="7" t="inlineStr">
         <is>
+          <t>KOMO 4 · KIRO 7 · KING 5 · KCPQ Fox 13</t>
+        </is>
+      </c>
+      <c r="K15" s="7" t="inlineStr">
+        <is>
+          <t>Bonneville (KIRO) · iHeart · Audacy</t>
+        </is>
+      </c>
+      <c r="L15" s="7" t="inlineStr">
+        <is>
+          <t>Wongdoody, Copacino Fujikado, DNA</t>
+        </is>
+      </c>
+      <c r="M15" s="7" t="inlineStr">
+        <is>
           <t>Billboard supply constrained by regulation; I-5/I-405 corridors strongest.</t>
         </is>
       </c>
@@ -54559,6 +54784,21 @@
       </c>
       <c r="J16" s="7" t="inlineStr">
         <is>
+          <t>KSTP 5 · WCCO 4 · KARE 11 · KMSP Fox 9</t>
+        </is>
+      </c>
+      <c r="K16" s="7" t="inlineStr">
+        <is>
+          <t>Hubbard (HQ — KSTP, KS95) · iHeart (KFAN) · Audacy (WCCO)</t>
+        </is>
+      </c>
+      <c r="L16" s="7" t="inlineStr">
+        <is>
+          <t>Fallon, Colle McVoy, Periscope</t>
+        </is>
+      </c>
+      <c r="M16" s="7" t="inlineStr">
+        <is>
           <t>Twin Cities; Franklin Outdoor runs 1,000+ illuminated boards across MN/W-WI.</t>
         </is>
       </c>
@@ -54605,6 +54845,21 @@
       </c>
       <c r="J17" s="7" t="inlineStr">
         <is>
+          <t>KNXV 15 · KPHO 5 · KPNX 12 · KSAZ Fox 10</t>
+        </is>
+      </c>
+      <c r="K17" s="7" t="inlineStr">
+        <is>
+          <t>Bonneville (KTAR) · iHeart · Hubbard</t>
+        </is>
+      </c>
+      <c r="L17" s="7" t="inlineStr">
+        <is>
+          <t>OH Partners, LaneTerralever, Zion &amp; Zion</t>
+        </is>
+      </c>
+      <c r="M17" s="7" t="inlineStr">
+        <is>
           <t>Freeway digital (Loop 101/202, I-10); sports-venue-adjacent units premium.</t>
         </is>
       </c>
@@ -54651,6 +54906,21 @@
       </c>
       <c r="J18" s="7" t="inlineStr">
         <is>
+          <t>WFTS 28 · WTSP 10 · WFLA 8 · WTVT Fox 13</t>
+        </is>
+      </c>
+      <c r="K18" s="7" t="inlineStr">
+        <is>
+          <t>iHeart (WFLA-AM) · Cox · Beasley (WQYK)</t>
+        </is>
+      </c>
+      <c r="L18" s="7" t="inlineStr">
+        <is>
+          <t>PPK, Schifino Lee</t>
+        </is>
+      </c>
+      <c r="M18" s="7" t="inlineStr">
+        <is>
           <t>Tampa Bay (Hillsborough/Pinellas); I-4 / I-275 / Veterans Expwy corridors.</t>
         </is>
       </c>
@@ -54697,6 +54967,21 @@
       </c>
       <c r="J19" s="7" t="inlineStr">
         <is>
+          <t>KMGH 7 · KCNC 4 · KUSA 9 · KDVR Fox 31</t>
+        </is>
+      </c>
+      <c r="K19" s="7" t="inlineStr">
+        <is>
+          <t>iHeart (KOA) · Bonneville (KYGO/KOSI) · Audacy</t>
+        </is>
+      </c>
+      <c r="L19" s="7" t="inlineStr">
+        <is>
+          <t>Karsh Hagan, Cactus, Grit Advertising</t>
+        </is>
+      </c>
+      <c r="M19" s="7" t="inlineStr">
+        <is>
           <t>I-25 / I-70 corridors; Mile High Outdoor runs 400+ metro displays.</t>
         </is>
       </c>
@@ -54743,6 +55028,21 @@
       </c>
       <c r="J20" s="7" t="inlineStr">
         <is>
+          <t>WEWS 5 · WOIO 19 · WKYC 3 · WJW Fox 8</t>
+        </is>
+      </c>
+      <c r="K20" s="7" t="inlineStr">
+        <is>
+          <t>iHeart (WTAM) · Audacy · Good Karma (WKNR)</t>
+        </is>
+      </c>
+      <c r="L20" s="7" t="inlineStr">
+        <is>
+          <t>Marcus Thomas, Adcom, Falls</t>
+        </is>
+      </c>
+      <c r="M20" s="7" t="inlineStr">
+        <is>
           <t>Cleveland/Akron/Canton; I-90 / I-77 / I-480 corridors; deep Ohio vendor stack.</t>
         </is>
       </c>
@@ -54789,6 +55089,21 @@
       </c>
       <c r="J21" s="7" t="inlineStr">
         <is>
+          <t>KXTV 10 · KOVR 13 · KCRA 3 · KTXL Fox 40</t>
+        </is>
+      </c>
+      <c r="K21" s="7" t="inlineStr">
+        <is>
+          <t>iHeart (KFBK) · Audacy · Bonneville</t>
+        </is>
+      </c>
+      <c r="L21" s="7" t="inlineStr">
+        <is>
+          <t>The Glass Agency, Position Interactive</t>
+        </is>
+      </c>
+      <c r="M21" s="7" t="inlineStr">
+        <is>
           <t>Sacramento/Stockton/Modesto DMA; Clear Channel runs 1,280+ displays across 5 counties.</t>
         </is>
       </c>
@@ -54835,6 +55150,21 @@
       </c>
       <c r="J22" s="7" t="inlineStr">
         <is>
+          <t>WFTV 9 · WKMG 6 · WESH 2 · WOFL Fox 35</t>
+        </is>
+      </c>
+      <c r="K22" s="7" t="inlineStr">
+        <is>
+          <t>iHeart · Cox (WDBO)</t>
+        </is>
+      </c>
+      <c r="L22" s="7" t="inlineStr">
+        <is>
+          <t>&amp;Barr, PUSH</t>
+        </is>
+      </c>
+      <c r="M22" s="7" t="inlineStr">
+        <is>
           <t>I-4 / theme-park &amp; tourist corridors carry premiums; strong visitor reach.</t>
         </is>
       </c>
@@ -54881,6 +55211,21 @@
       </c>
       <c r="J23" s="7" t="inlineStr">
         <is>
+          <t>KDNL 30 · KMOV 4 · KSDK 5 · KTVI Fox 2</t>
+        </is>
+      </c>
+      <c r="K23" s="7" t="inlineStr">
+        <is>
+          <t>Audacy (KMOX) · iHeart · Hubbard</t>
+        </is>
+      </c>
+      <c r="L23" s="7" t="inlineStr">
+        <is>
+          <t>HLK, Rodgers Townsend (DDB)</t>
+        </is>
+      </c>
+      <c r="M23" s="7" t="inlineStr">
+        <is>
           <t>Bi-state (MO/IL); DDI Media the dominant independent along I-70 and the Illinois side.</t>
         </is>
       </c>
@@ -54927,6 +55272,21 @@
       </c>
       <c r="J24" s="7" t="inlineStr">
         <is>
+          <t>WTAE 4 · KDKA 2 · WPXI 11 · WPGH Fox 53</t>
+        </is>
+      </c>
+      <c r="K24" s="7" t="inlineStr">
+        <is>
+          <t>Audacy (KDKA) · iHeart (WDVE) · Steel City Media</t>
+        </is>
+      </c>
+      <c r="L24" s="7" t="inlineStr">
+        <is>
+          <t>Brunner, MARC USA (legacy), Gatesman</t>
+        </is>
+      </c>
+      <c r="M24" s="7" t="inlineStr">
+        <is>
           <t>Parkway/tunnel approaches; strong independent scene (TM, Penneco, Steel City).</t>
         </is>
       </c>
@@ -54973,6 +55333,21 @@
       </c>
       <c r="J25" s="7" t="inlineStr">
         <is>
+          <t>KGTV 10 · KFMB 8 · KNSD 7/39 · KSWB Fox 5</t>
+        </is>
+      </c>
+      <c r="K25" s="7" t="inlineStr">
+        <is>
+          <t>iHeart (KOGO) · Audacy · Local Media San Diego</t>
+        </is>
+      </c>
+      <c r="L25" s="7" t="inlineStr">
+        <is>
+          <t>VITRO (Petco work), i.d.e.a.</t>
+        </is>
+      </c>
+      <c r="M25" s="7" t="inlineStr">
+        <is>
           <t>I-5 / I-805 / I-15 / Hwy-78 corridors; limited inventory keeps rates firm.</t>
         </is>
       </c>
@@ -55019,6 +55394,21 @@
       </c>
       <c r="J26" s="7" t="inlineStr">
         <is>
+          <t>WMAR 2 · WJZ 13 · WBAL 11 · WBFF Fox 45</t>
+        </is>
+      </c>
+      <c r="K26" s="7" t="inlineStr">
+        <is>
+          <t>Hearst (WBAL radio) · iHeart · Audacy</t>
+        </is>
+      </c>
+      <c r="L26" s="7" t="inlineStr">
+        <is>
+          <t>Planit, GKV, idfive</t>
+        </is>
+      </c>
+      <c r="M26" s="7" t="inlineStr">
+        <is>
           <t>I-95 / I-695 Beltway; Vision Outdoor is the Mid-Atlantic's independent digital operator.</t>
         </is>
       </c>
@@ -55065,6 +55455,21 @@
       </c>
       <c r="J27" s="7" t="inlineStr">
         <is>
+          <t>WSOC 9 · WBTV 3 · WCNC 36 · WJZY Fox 46</t>
+        </is>
+      </c>
+      <c r="K27" s="7" t="inlineStr">
+        <is>
+          <t>iHeart · Urban One · Norsan Media (Spanish, local)</t>
+        </is>
+      </c>
+      <c r="L27" s="7" t="inlineStr">
+        <is>
+          <t>Wray Ward, Luquire</t>
+        </is>
+      </c>
+      <c r="M27" s="7" t="inlineStr">
+        <is>
           <t>I-77 / I-85 / I-485 corridors; Adams Outdoor reaches 1.8M across 22 counties.</t>
         </is>
       </c>
@@ -55111,6 +55516,21 @@
       </c>
       <c r="J28" s="7" t="inlineStr">
         <is>
+          <t>WTVD 11 · WNCN 17 · WRAL 5 · WRAZ Fox 50</t>
+        </is>
+      </c>
+      <c r="K28" s="7" t="inlineStr">
+        <is>
+          <t>iHeart · Curtis Media (local Triangle) · Capitol Broadcasting</t>
+        </is>
+      </c>
+      <c r="L28" s="7" t="inlineStr">
+        <is>
+          <t>McKinney (Durham), Baldwin&amp;</t>
+        </is>
+      </c>
+      <c r="M28" s="7" t="inlineStr">
+        <is>
           <t>Research Triangle; I-40 / I-440 Beltline; Adams/Allison/Trailhead active regionally.</t>
         </is>
       </c>
@@ -55157,6 +55577,21 @@
       </c>
       <c r="J29" s="7" t="inlineStr">
         <is>
+          <t>WRTV 6 · WTTV 4 · WTHR 13 · WXIN Fox 59</t>
+        </is>
+      </c>
+      <c r="K29" s="7" t="inlineStr">
+        <is>
+          <t>iHeart · Cumulus (WFMS) · Urban One</t>
+        </is>
+      </c>
+      <c r="L29" s="7" t="inlineStr">
+        <is>
+          <t>Young &amp; Laramore, Hirons</t>
+        </is>
+      </c>
+      <c r="M29" s="7" t="inlineStr">
+        <is>
           <t>'Crossroads of America' — I-65/I-70/I-465; Lamar-dominant plus Keyes &amp; Reagan.</t>
         </is>
       </c>
@@ -55203,6 +55638,21 @@
       </c>
       <c r="J30" s="7" t="inlineStr">
         <is>
+          <t>WCPO 9 · WKRC 12 · WLWT 5 · WXIX Fox 19</t>
+        </is>
+      </c>
+      <c r="K30" s="7" t="inlineStr">
+        <is>
+          <t>iHeart (700WLW) · Hubbard (WKRQ) · Cumulus</t>
+        </is>
+      </c>
+      <c r="L30" s="7" t="inlineStr">
+        <is>
+          <t>Curiosity, Barefoot Proximity (BBDO)</t>
+        </is>
+      </c>
+      <c r="M30" s="7" t="inlineStr">
+        <is>
           <t>I-71 / I-75 / I-275 loop; tri-state (OH/KY/IN); Lamar &amp; Key-Ads strong.</t>
         </is>
       </c>
@@ -55249,6 +55699,21 @@
       </c>
       <c r="J31" s="7" t="inlineStr">
         <is>
+          <t>KTNV 13 · KLAS 8 · KSNV 3 · KVVU Fox 5</t>
+        </is>
+      </c>
+      <c r="K31" s="7" t="inlineStr">
+        <is>
+          <t>Audacy · iHeart · Lotus (local)</t>
+        </is>
+      </c>
+      <c r="L31" s="7" t="inlineStr">
+        <is>
+          <t>R&amp;R Partners ('What happens here, stays here')</t>
+        </is>
+      </c>
+      <c r="M31" s="7" t="inlineStr">
+        <is>
           <t>The Strip commands outsized rates (spectaculars far higher); OUTFRONT reaches 99.9% weekly.</t>
         </is>
       </c>
@@ -55295,6 +55760,21 @@
       </c>
       <c r="J32" s="7" t="inlineStr">
         <is>
+          <t>KSAT 12 · KENS 5 · WOAI 4 · KABB Fox 29</t>
+        </is>
+      </c>
+      <c r="K32" s="7" t="inlineStr">
+        <is>
+          <t>iHeartMedia (corporate HQ — WOAI) · Cox · Univision (Spanish)</t>
+        </is>
+      </c>
+      <c r="L32" s="7" t="inlineStr">
+        <is>
+          <t>The Atkins Group, Giles-Parscale (legacy)</t>
+        </is>
+      </c>
+      <c r="M32" s="7" t="inlineStr">
+        <is>
           <t>I-10 / Loop 410 / US-281 the strongest placements.</t>
         </is>
       </c>
@@ -55341,6 +55821,21 @@
       </c>
       <c r="J33" s="7" t="inlineStr">
         <is>
+          <t>KATU 2 · KOIN 6 · KGW 8 · KPTV Fox 12</t>
+        </is>
+      </c>
+      <c r="K33" s="7" t="inlineStr">
+        <is>
+          <t>iHeart (KEX) · Audacy · Alpha Media (HQ Portland)</t>
+        </is>
+      </c>
+      <c r="L33" s="7" t="inlineStr">
+        <is>
+          <t>Wieden+Kennedy (HQ), Instrument, Opinionated</t>
+        </is>
+      </c>
+      <c r="M33" s="7" t="inlineStr">
+        <is>
           <t>Lamar is the largest footprint + sole PDX operator; wallscapes in the Pearl/Downtown.</t>
         </is>
       </c>
@@ -55387,6 +55882,21 @@
       </c>
       <c r="J34" s="7" t="inlineStr">
         <is>
+          <t>WISN 12 · WDJT 58 · WTMJ 4 · WITI Fox 6</t>
+        </is>
+      </c>
+      <c r="K34" s="7" t="inlineStr">
+        <is>
+          <t>Good Karma (WTMJ radio) · iHeart · Saga (WKLH)</t>
+        </is>
+      </c>
+      <c r="L34" s="7" t="inlineStr">
+        <is>
+          <t>Cramer-Krasselt, BVK, Hoffman York</t>
+        </is>
+      </c>
+      <c r="M34" s="7" t="inlineStr">
+        <is>
           <t>I-94 / I-43 corridors; Lamar-dominant plus regional Ohio/Wisconsin operators.</t>
         </is>
       </c>
@@ -55433,6 +55943,21 @@
       </c>
       <c r="J35" s="7" t="inlineStr">
         <is>
+          <t>WSYX 6 · WBNS 10 · WCMH 4 · WTTE Fox 28</t>
+        </is>
+      </c>
+      <c r="K35" s="7" t="inlineStr">
+        <is>
+          <t>iHeart (WTVN/WNCI) · Saga (WSNY) · Urban One</t>
+        </is>
+      </c>
+      <c r="L35" s="7" t="inlineStr">
+        <is>
+          <t>Fahlgren Mortine, The Shipyard, Ologie</t>
+        </is>
+      </c>
+      <c r="M35" s="7" t="inlineStr">
+        <is>
           <t>~2,200 boards; one of the Midwest's deepest OOH inventories (OAA of Ohio HQ'd here).</t>
         </is>
       </c>
@@ -55479,6 +56004,21 @@
       </c>
       <c r="J36" s="7" t="inlineStr">
         <is>
+          <t>KMBC 9 · KCTV 5 · KSHB 41 · WDAF Fox 4</t>
+        </is>
+      </c>
+      <c r="K36" s="7" t="inlineStr">
+        <is>
+          <t>Audacy (KMBZ) · Cumulus · Carter Broadcast (KPRS)</t>
+        </is>
+      </c>
+      <c r="L36" s="7" t="inlineStr">
+        <is>
+          <t>VML (HQ), Barkley OKRP</t>
+        </is>
+      </c>
+      <c r="M36" s="7" t="inlineStr">
+        <is>
           <t>I-35/I-70; Ad-Trend the largest locally owned operator (since 1985).</t>
         </is>
       </c>
@@ -55525,6 +56065,21 @@
       </c>
       <c r="J37" s="7" t="inlineStr">
         <is>
+          <t>WKRN 2 · WTVF 5 · WSMV 4 · WZTV Fox 17</t>
+        </is>
+      </c>
+      <c r="K37" s="7" t="inlineStr">
+        <is>
+          <t>iHeart (WLAC) · Cumulus (WKDF/WSM-FM) · Opry Ent. (WSM-AM)</t>
+        </is>
+      </c>
+      <c r="L37" s="7" t="inlineStr">
+        <is>
+          <t>bohan, GS&amp;F</t>
+        </is>
+      </c>
+      <c r="M37" s="7" t="inlineStr">
+        <is>
           <t>I-40 / I-24 / I-65 and Broadway/tourism demand; Allison Outdoor active regionally.</t>
         </is>
       </c>
@@ -55571,6 +56126,21 @@
       </c>
       <c r="J38" s="7" t="inlineStr">
         <is>
+          <t>KTVX 4 · KUTV 2 · KSL 5 · KSTU Fox 13</t>
+        </is>
+      </c>
+      <c r="K38" s="7" t="inlineStr">
+        <is>
+          <t>Bonneville (HQ — KSL) · iHeart · Broadway Media (local)</t>
+        </is>
+      </c>
+      <c r="L38" s="7" t="inlineStr">
+        <is>
+          <t>Struck, Love Communications, Richter7</t>
+        </is>
+      </c>
+      <c r="M38" s="7" t="inlineStr">
+        <is>
           <t>I-15 corridor; Reagan Outdoor (HQ) &amp; YESCO dominate; billboards politically restricted.</t>
         </is>
       </c>
@@ -55617,6 +56187,21 @@
       </c>
       <c r="J39" s="7" t="inlineStr">
         <is>
+          <t>WGNO 26 · WWL 4 · WDSU 6 · WVUE Fox 8</t>
+        </is>
+      </c>
+      <c r="K39" s="7" t="inlineStr">
+        <is>
+          <t>Audacy (WWL radio) · iHeart · Cumulus</t>
+        </is>
+      </c>
+      <c r="L39" s="7" t="inlineStr">
+        <is>
+          <t>Peter Mayer, Trumpet</t>
+        </is>
+      </c>
+      <c r="M39" s="7" t="inlineStr">
+        <is>
           <t>I-10 / French Quarter &amp; tourism demand; Lamar (Louisiana roots) &amp; Lindmark strong.</t>
         </is>
       </c>
@@ -55663,6 +56248,21 @@
       </c>
       <c r="J40" s="7" t="inlineStr">
         <is>
+          <t>KOCO 5 · KWTV 9 · KFOR 4 · KOKH Fox 25</t>
+        </is>
+      </c>
+      <c r="K40" s="7" t="inlineStr">
+        <is>
+          <t>iHeart (KTOK) · Cumulus (KATT) · Tyler Media (local)</t>
+        </is>
+      </c>
+      <c r="L40" s="7" t="inlineStr">
+        <is>
+          <t>Ackerman McQueen, VI Marketing + Branding</t>
+        </is>
+      </c>
+      <c r="M40" s="7" t="inlineStr">
+        <is>
           <t>I-35 / I-40 / I-44; Lindmark, Headrick and BM cover Oklahoma broadly.</t>
         </is>
       </c>
@@ -55709,6 +56309,21 @@
       </c>
       <c r="J41" s="7" t="inlineStr">
         <is>
+          <t>WATN 24 · WREG 3 · WMC 5 · WHBQ Fox 13</t>
+        </is>
+      </c>
+      <c r="K41" s="7" t="inlineStr">
+        <is>
+          <t>iHeart · Cumulus · Flinn Broadcasting (local)</t>
+        </is>
+      </c>
+      <c r="L41" s="7" t="inlineStr">
+        <is>
+          <t>archer malmo (Signet), Sullivan Branding</t>
+        </is>
+      </c>
+      <c r="M41" s="7" t="inlineStr">
+        <is>
           <t>I-40 / I-55 freight corridors; Lamar-dominant plus Allison Outdoor regionally.</t>
         </is>
       </c>
@@ -55755,6 +56370,21 @@
       </c>
       <c r="J42" s="7" t="inlineStr">
         <is>
+          <t>WRIC 8 · WTVR 6 · WWBT 12 · WRLH Fox 35</t>
+        </is>
+      </c>
+      <c r="K42" s="7" t="inlineStr">
+        <is>
+          <t>Audacy (WRVA) · SummitMedia · Urban One</t>
+        </is>
+      </c>
+      <c r="L42" s="7" t="inlineStr">
+        <is>
+          <t>The Martin Agency (GEICO), Arts &amp; Letters</t>
+        </is>
+      </c>
+      <c r="M42" s="7" t="inlineStr">
+        <is>
           <t>I-95 / I-64 corridors; Lamar &amp; OUTFRONT dominant in a supply-limited market.</t>
         </is>
       </c>
@@ -55801,6 +56431,21 @@
       </c>
       <c r="J43" s="7" t="inlineStr">
         <is>
+          <t>KVUE 24 · KEYE 42 · KXAN 36 · KTBC Fox 7</t>
+        </is>
+      </c>
+      <c r="K43" s="7" t="inlineStr">
+        <is>
+          <t>iHeart · Audacy · Waterloo Media (local — KLBJ)</t>
+        </is>
+      </c>
+      <c r="L43" s="7" t="inlineStr">
+        <is>
+          <t>GSD&amp;M (HQ), McGarrah Jessee, Preacher</t>
+        </is>
+      </c>
+      <c r="M43" s="7" t="inlineStr">
+        <is>
           <t>Reagan Outdoor-dominated; tech-driven demand along I-35 / MoPac / US-183.</t>
         </is>
       </c>
@@ -55847,14 +56492,29 @@
       </c>
       <c r="J44" s="7" t="inlineStr">
         <is>
+          <t>WJXX 25 · WJAX 47 · WTLV 12 · WFOX 30</t>
+        </is>
+      </c>
+      <c r="K44" s="7" t="inlineStr">
+        <is>
+          <t>Cox (WOKV/WAPE) · iHeart</t>
+        </is>
+      </c>
+      <c r="L44" s="7" t="inlineStr">
+        <is>
+          <t>Dalton Agency, Shepherd (St. John &amp; Partners)</t>
+        </is>
+      </c>
+      <c r="M44" s="7" t="inlineStr">
+        <is>
           <t>Largest US city by land area; I-95 / I-295 corridors carry the value.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A2:J44"/>
+  <autoFilter ref="A2:M44"/>
   <mergeCells count="1">
-    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A1:M1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -63894,6 +64554,1995 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:I46"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="38" customWidth="1" min="5" max="5"/>
+    <col width="34" customWidth="1" min="6" max="6"/>
+    <col width="36" customWidth="1" min="7" max="7"/>
+    <col width="28" customWidth="1" min="8" max="8"/>
+    <col width="34" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>US QUICK-START BY METRO - WHO TO CALL IN EACH MARKET</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="n"/>
+      <c r="C1" s="2" t="n"/>
+      <c r="D1" s="2" t="n"/>
+      <c r="E1" s="2" t="n"/>
+      <c r="F1" s="2" t="n"/>
+      <c r="G1" s="2" t="n"/>
+      <c r="H1" s="2" t="n"/>
+      <c r="I1" s="2" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>Rank</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>Metro</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>Metro Pop</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>OOH Rate Band</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="inlineStr">
+        <is>
+          <t>Top Local OOH Operators</t>
+        </is>
+      </c>
+      <c r="F2" s="5" t="inlineStr">
+        <is>
+          <t>Big-4 TV</t>
+        </is>
+      </c>
+      <c r="G2" s="5" t="inlineStr">
+        <is>
+          <t>Radio Groups</t>
+        </is>
+      </c>
+      <c r="H2" s="5" t="inlineStr">
+        <is>
+          <t>Newspaper</t>
+        </is>
+      </c>
+      <c r="I2" s="5" t="inlineStr">
+        <is>
+          <t>Agencies to Call</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>New York</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>19.9M</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>$3,000-$50,000/mo</t>
+        </is>
+      </c>
+      <c r="E3" s="7" t="inlineStr">
+        <is>
+          <t>JCDecaux, Branded Cities Network, Brooklyn Outdoor</t>
+        </is>
+      </c>
+      <c r="F3" s="7" t="inlineStr">
+        <is>
+          <t>WABC 7 · WCBS 2 · WNBC 4 · WNYW Fox 5</t>
+        </is>
+      </c>
+      <c r="G3" s="7" t="inlineStr">
+        <is>
+          <t>Audacy (WFAN, 1010 WINS) · iHeart (Z100) · SBS (Spanish, HQ)</t>
+        </is>
+      </c>
+      <c r="H3" s="7" t="inlineStr">
+        <is>
+          <t>The New York Times / NY Post / Daily News</t>
+        </is>
+      </c>
+      <c r="I3" s="7" t="inlineStr">
+        <is>
+          <t>Ogilvy, BBDO, Droga5, McCann (global HQs)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>Los Angeles</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>13.0M</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>$2,500-$40,000/mo</t>
+        </is>
+      </c>
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>JCDecaux, Regency Outdoor Advertising, Branded Cities Network</t>
+        </is>
+      </c>
+      <c r="F4" s="7" t="inlineStr">
+        <is>
+          <t>KABC 7 · KCBS 2 · KNBC 4 · KTTV Fox 11</t>
+        </is>
+      </c>
+      <c r="G4" s="7" t="inlineStr">
+        <is>
+          <t>iHeart (KIIS, KFI) · Audacy (KROQ, KNX) · Univision/SBS (Spanish)</t>
+        </is>
+      </c>
+      <c r="H4" s="7" t="inlineStr">
+        <is>
+          <t>Los Angeles Times</t>
+        </is>
+      </c>
+      <c r="I4" s="7" t="inlineStr">
+        <is>
+          <t>Deutsch LA, 72andSunny, TBWA\Chiat\Day</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>Chicago</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>9.4M</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>$2,000-$25,000/mo</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>JCDecaux, Becker Boards, Branded Cities Network</t>
+        </is>
+      </c>
+      <c r="F5" s="7" t="inlineStr">
+        <is>
+          <t>WLS 7 · WBBM 2 · WMAQ 5 · WFLD Fox 32</t>
+        </is>
+      </c>
+      <c r="G5" s="7" t="inlineStr">
+        <is>
+          <t>Audacy (WBBM, WSCR) · iHeart · Nexstar (WGN Radio)</t>
+        </is>
+      </c>
+      <c r="H5" s="7" t="inlineStr">
+        <is>
+          <t>Chicago Tribune / Sun-Times</t>
+        </is>
+      </c>
+      <c r="I5" s="7" t="inlineStr">
+        <is>
+          <t>Leo Burnett, FCB Chicago, Energy BBDO</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>San Francisco</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>4.6M (Bay CSA ~9.7M)</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>$2,500-$30,000/mo</t>
+        </is>
+      </c>
+      <c r="E6" s="7" t="inlineStr">
+        <is>
+          <t>Becker Boards</t>
+        </is>
+      </c>
+      <c r="F6" s="7" t="inlineStr">
+        <is>
+          <t>KGO 7 · KPIX 5 · KNTV 11 · KTVU Fox 2</t>
+        </is>
+      </c>
+      <c r="G6" s="7" t="inlineStr">
+        <is>
+          <t>Audacy (KCBS) · iHeart · Bonneville</t>
+        </is>
+      </c>
+      <c r="H6" s="7" t="inlineStr">
+        <is>
+          <t>San Francisco Chronicle</t>
+        </is>
+      </c>
+      <c r="I6" s="7" t="inlineStr">
+        <is>
+          <t>Goodby Silverstein, Duncan Channon, Argonaut</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>Atlanta</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>6.4M</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>$1,500-$16,000/mo</t>
+        </is>
+      </c>
+      <c r="E7" s="7" t="inlineStr">
+        <is>
+          <t>Adams Outdoor Advertising, Billboard Company Atlanta, Trailhead Media</t>
+        </is>
+      </c>
+      <c r="F7" s="7" t="inlineStr">
+        <is>
+          <t>WSB 2 · WANF 46 · WXIA 11 · WAGA Fox 5</t>
+        </is>
+      </c>
+      <c r="G7" s="7" t="inlineStr">
+        <is>
+          <t>Cox Media Group (HQ, WSB) · iHeart · Urban One</t>
+        </is>
+      </c>
+      <c r="H7" s="7" t="inlineStr">
+        <is>
+          <t>The Atlanta Journal-Constitution</t>
+        </is>
+      </c>
+      <c r="I7" s="7" t="inlineStr">
+        <is>
+          <t>22squared, Dagger, Chemistry</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>Washington DC</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>6.3M</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>$2,000-$20,000/mo</t>
+        </is>
+      </c>
+      <c r="E8" s="7" t="inlineStr">
+        <is>
+          <t>Capitol Outdoor, Digital Outdoor Advertising, LLC, Digital Outdoor Advertising — DC</t>
+        </is>
+      </c>
+      <c r="F8" s="7" t="inlineStr">
+        <is>
+          <t>WJLA 7 · WUSA 9 · WRC 4 · WTTG Fox 5</t>
+        </is>
+      </c>
+      <c r="G8" s="7" t="inlineStr">
+        <is>
+          <t>Hubbard (WTOP — top-billing US station) · iHeart · Cumulus (WMAL)</t>
+        </is>
+      </c>
+      <c r="H8" s="7" t="inlineStr">
+        <is>
+          <t>The Washington Post</t>
+        </is>
+      </c>
+      <c r="I8" s="7" t="inlineStr">
+        <is>
+          <t>GMMB (political), RP3 Agency</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>Boston</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>4.9M</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>$1,800-$18,000/mo</t>
+        </is>
+      </c>
+      <c r="E9" s="7" t="inlineStr">
+        <is>
+          <t>Digital Outdoor Advertising, LLC</t>
+        </is>
+      </c>
+      <c r="F9" s="7" t="inlineStr">
+        <is>
+          <t>WCVB 5 · WBZ 4 · WBTS 10 · WFXT Fox 25</t>
+        </is>
+      </c>
+      <c r="G9" s="7" t="inlineStr">
+        <is>
+          <t>iHeart (WBZ-AM) · Audacy (WEEI) · Beasley</t>
+        </is>
+      </c>
+      <c r="H9" s="7" t="inlineStr">
+        <is>
+          <t>The Boston Globe</t>
+        </is>
+      </c>
+      <c r="I9" s="7" t="inlineStr">
+        <is>
+          <t>Hill Holliday, Arnold, MullenLowe, Allen &amp; Gerritsen</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>Dallas</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>8.1M</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>$1,500-$18,000/mo</t>
+        </is>
+      </c>
+      <c r="E10" s="7" t="inlineStr">
+        <is>
+          <t>SignAd Outdoor Advertising, Arrington Outdoor Advertising, Lux Media</t>
+        </is>
+      </c>
+      <c r="F10" s="7" t="inlineStr">
+        <is>
+          <t>WFAA 8 · KTVT 11 · KXAS 5 · KDFW Fox 4</t>
+        </is>
+      </c>
+      <c r="G10" s="7" t="inlineStr">
+        <is>
+          <t>iHeart · Audacy (KRLD) · Cumulus (WBAP)</t>
+        </is>
+      </c>
+      <c r="H10" s="7" t="inlineStr">
+        <is>
+          <t>The Dallas Morning News</t>
+        </is>
+      </c>
+      <c r="I10" s="7" t="inlineStr">
+        <is>
+          <t>TRG (The Richards Group), Dieste (Hispanic)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>Houston</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>7.5M</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>$1,500-$15,000/mo</t>
+        </is>
+      </c>
+      <c r="E11" s="7" t="inlineStr">
+        <is>
+          <t>SignAd Outdoor Advertising, Gilbreath Outdoor Advertising, Lux Media</t>
+        </is>
+      </c>
+      <c r="F11" s="7" t="inlineStr">
+        <is>
+          <t>KTRK 13 · KHOU 11 · KPRC 2 · KRIV Fox 26</t>
+        </is>
+      </c>
+      <c r="G11" s="7" t="inlineStr">
+        <is>
+          <t>iHeart (KTRH) · Audacy · Cox (KKBQ)</t>
+        </is>
+      </c>
+      <c r="H11" s="7" t="inlineStr">
+        <is>
+          <t>Houston Chronicle</t>
+        </is>
+      </c>
+      <c r="I11" s="7" t="inlineStr">
+        <is>
+          <t>Lopez Negrete (Hispanic), MMI Agency</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>Miami</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>6.2M</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="inlineStr">
+        <is>
+          <t>$1,800-$20,000/mo</t>
+        </is>
+      </c>
+      <c r="E12" s="7" t="inlineStr">
+        <is>
+          <t>Becker Boards, Capitol Outdoor, Carter Outdoor Advertising</t>
+        </is>
+      </c>
+      <c r="F12" s="7" t="inlineStr">
+        <is>
+          <t>WPLG 10 · WFOR 4 · WTVJ 6 · WSVN Fox 7</t>
+        </is>
+      </c>
+      <c r="G12" s="7" t="inlineStr">
+        <is>
+          <t>iHeart · Cox · SBS (Spanish broadcasting HQ)</t>
+        </is>
+      </c>
+      <c r="H12" s="7" t="inlineStr">
+        <is>
+          <t>Miami Herald</t>
+        </is>
+      </c>
+      <c r="I12" s="7" t="inlineStr">
+        <is>
+          <t>Zimmerman, Crispin (legacy), República Havas (Hispanic)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>Philadelphia</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>6.2M</t>
+        </is>
+      </c>
+      <c r="D13" s="6" t="inlineStr">
+        <is>
+          <t>$1,500-$12,000/mo</t>
+        </is>
+      </c>
+      <c r="E13" s="7" t="inlineStr">
+        <is>
+          <t>Capitol Outdoor, Digital Outdoor Advertising, LLC, Intersection</t>
+        </is>
+      </c>
+      <c r="F13" s="7" t="inlineStr">
+        <is>
+          <t>WPVI 6 · KYW 3 · WCAU 10 · WTXF Fox 29</t>
+        </is>
+      </c>
+      <c r="G13" s="7" t="inlineStr">
+        <is>
+          <t>Audacy (HQ — KYW, WIP) · iHeart · Beasley (WMMR)</t>
+        </is>
+      </c>
+      <c r="H13" s="7" t="inlineStr">
+        <is>
+          <t>The Philadelphia Inquirer</t>
+        </is>
+      </c>
+      <c r="I13" s="7" t="inlineStr">
+        <is>
+          <t>Digitas Philly (legacy), Brownstein Group, LevLane</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>Detroit</t>
+        </is>
+      </c>
+      <c r="C14" s="6" t="inlineStr">
+        <is>
+          <t>4.3M</t>
+        </is>
+      </c>
+      <c r="D14" s="6" t="inlineStr">
+        <is>
+          <t>$1,200-$12,000/mo</t>
+        </is>
+      </c>
+      <c r="E14" s="7" t="inlineStr">
+        <is>
+          <t>International Outdoor</t>
+        </is>
+      </c>
+      <c r="F14" s="7" t="inlineStr">
+        <is>
+          <t>WXYZ 7 · WWJ 62 · WDIV 4 · WJBK Fox 2</t>
+        </is>
+      </c>
+      <c r="G14" s="7" t="inlineStr">
+        <is>
+          <t>Audacy (WWJ, WXYT) · iHeart · Cumulus (WJR)</t>
+        </is>
+      </c>
+      <c r="H14" s="7" t="inlineStr">
+        <is>
+          <t>Detroit Free Press / The Detroit News</t>
+        </is>
+      </c>
+      <c r="I14" s="7" t="inlineStr">
+        <is>
+          <t>Doner, Campbell Ewald, Lafayette American</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>Seattle</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>4.0M</t>
+        </is>
+      </c>
+      <c r="D15" s="6" t="inlineStr">
+        <is>
+          <t>$1,500-$14,000/mo</t>
+        </is>
+      </c>
+      <c r="E15" s="7" t="inlineStr">
+        <is>
+          <t>Pacific Outdoor Advertising, Parker Outdoor Inc., Summus Outdoor</t>
+        </is>
+      </c>
+      <c r="F15" s="7" t="inlineStr">
+        <is>
+          <t>KOMO 4 · KIRO 7 · KING 5 · KCPQ Fox 13</t>
+        </is>
+      </c>
+      <c r="G15" s="7" t="inlineStr">
+        <is>
+          <t>Bonneville (KIRO) · iHeart · Audacy</t>
+        </is>
+      </c>
+      <c r="H15" s="7" t="inlineStr">
+        <is>
+          <t>The Seattle Times</t>
+        </is>
+      </c>
+      <c r="I15" s="7" t="inlineStr">
+        <is>
+          <t>Wongdoody, Copacino Fujikado, DNA</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>Minneapolis</t>
+        </is>
+      </c>
+      <c r="C16" s="6" t="inlineStr">
+        <is>
+          <t>3.7M</t>
+        </is>
+      </c>
+      <c r="D16" s="6" t="inlineStr">
+        <is>
+          <t>$1,200-$12,000/mo</t>
+        </is>
+      </c>
+      <c r="E16" s="7" t="inlineStr">
+        <is>
+          <t>Franklin Outdoor Advertising, Blue Ox Media</t>
+        </is>
+      </c>
+      <c r="F16" s="7" t="inlineStr">
+        <is>
+          <t>KSTP 5 · WCCO 4 · KARE 11 · KMSP Fox 9</t>
+        </is>
+      </c>
+      <c r="G16" s="7" t="inlineStr">
+        <is>
+          <t>Hubbard (HQ — KSTP, KS95) · iHeart (KFAN) · Audacy (WCCO)</t>
+        </is>
+      </c>
+      <c r="H16" s="7" t="inlineStr">
+        <is>
+          <t>Star Tribune</t>
+        </is>
+      </c>
+      <c r="I16" s="7" t="inlineStr">
+        <is>
+          <t>Fallon, Colle McVoy, Periscope</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>Phoenix</t>
+        </is>
+      </c>
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>5.1M</t>
+        </is>
+      </c>
+      <c r="D17" s="6" t="inlineStr">
+        <is>
+          <t>$1,200-$10,000/mo</t>
+        </is>
+      </c>
+      <c r="E17" s="7" t="inlineStr">
+        <is>
+          <t>American Outdoor Advertising, Arizona Billboard Company, Becker Boards</t>
+        </is>
+      </c>
+      <c r="F17" s="7" t="inlineStr">
+        <is>
+          <t>KNXV 15 · KPHO 5 · KPNX 12 · KSAZ Fox 10</t>
+        </is>
+      </c>
+      <c r="G17" s="7" t="inlineStr">
+        <is>
+          <t>Bonneville (KTAR) · iHeart · Hubbard</t>
+        </is>
+      </c>
+      <c r="H17" s="7" t="inlineStr">
+        <is>
+          <t>The Arizona Republic</t>
+        </is>
+      </c>
+      <c r="I17" s="7" t="inlineStr">
+        <is>
+          <t>OH Partners, LaneTerralever, Zion &amp; Zion</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>Tampa</t>
+        </is>
+      </c>
+      <c r="C18" s="6" t="inlineStr">
+        <is>
+          <t>3.3M</t>
+        </is>
+      </c>
+      <c r="D18" s="6" t="inlineStr">
+        <is>
+          <t>$1,200-$11,000/mo</t>
+        </is>
+      </c>
+      <c r="E18" s="7" t="inlineStr">
+        <is>
+          <t>Tampa Outdoor Advertising, Logan Outdoor Advertising, Signal Outdoor Advertising</t>
+        </is>
+      </c>
+      <c r="F18" s="7" t="inlineStr">
+        <is>
+          <t>WFTS 28 · WTSP 10 · WFLA 8 · WTVT Fox 13</t>
+        </is>
+      </c>
+      <c r="G18" s="7" t="inlineStr">
+        <is>
+          <t>iHeart (WFLA-AM) · Cox · Beasley (WQYK)</t>
+        </is>
+      </c>
+      <c r="H18" s="7" t="inlineStr">
+        <is>
+          <t>Tampa Bay Times</t>
+        </is>
+      </c>
+      <c r="I18" s="7" t="inlineStr">
+        <is>
+          <t>PPK, Schifino Lee</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="n">
+        <v>17</v>
+      </c>
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>Denver</t>
+        </is>
+      </c>
+      <c r="C19" s="6" t="inlineStr">
+        <is>
+          <t>3.0M</t>
+        </is>
+      </c>
+      <c r="D19" s="6" t="inlineStr">
+        <is>
+          <t>$1,200-$11,000/mo</t>
+        </is>
+      </c>
+      <c r="E19" s="7" t="inlineStr">
+        <is>
+          <t>Mile High Outdoor, Elevation Outdoor Advertising, Outdoor Ads, Inc.</t>
+        </is>
+      </c>
+      <c r="F19" s="7" t="inlineStr">
+        <is>
+          <t>KMGH 7 · KCNC 4 · KUSA 9 · KDVR Fox 31</t>
+        </is>
+      </c>
+      <c r="G19" s="7" t="inlineStr">
+        <is>
+          <t>iHeart (KOA) · Bonneville (KYGO/KOSI) · Audacy</t>
+        </is>
+      </c>
+      <c r="H19" s="7" t="inlineStr">
+        <is>
+          <t>The Denver Post</t>
+        </is>
+      </c>
+      <c r="I19" s="7" t="inlineStr">
+        <is>
+          <t>Karsh Hagan, Cactus, Grit Advertising</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="B20" s="7" t="inlineStr">
+        <is>
+          <t>Cleveland</t>
+        </is>
+      </c>
+      <c r="C20" s="6" t="inlineStr">
+        <is>
+          <t>2.2M</t>
+        </is>
+      </c>
+      <c r="D20" s="6" t="inlineStr">
+        <is>
+          <t>$1,000-$11,000/mo</t>
+        </is>
+      </c>
+      <c r="E20" s="7" t="inlineStr">
+        <is>
+          <t>American Outdoor Advertising (Columbus), Outdoor Advertising Center, Key-Ads, Inc.</t>
+        </is>
+      </c>
+      <c r="F20" s="7" t="inlineStr">
+        <is>
+          <t>WEWS 5 · WOIO 19 · WKYC 3 · WJW Fox 8</t>
+        </is>
+      </c>
+      <c r="G20" s="7" t="inlineStr">
+        <is>
+          <t>iHeart (WTAM) · Audacy · Good Karma (WKNR)</t>
+        </is>
+      </c>
+      <c r="H20" s="7" t="inlineStr">
+        <is>
+          <t>The Plain Dealer / cleveland.com</t>
+        </is>
+      </c>
+      <c r="I20" s="7" t="inlineStr">
+        <is>
+          <t>Marcus Thomas, Adcom, Falls</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="B21" s="7" t="inlineStr">
+        <is>
+          <t>Sacramento</t>
+        </is>
+      </c>
+      <c r="C21" s="6" t="inlineStr">
+        <is>
+          <t>2.4M</t>
+        </is>
+      </c>
+      <c r="D21" s="6" t="inlineStr">
+        <is>
+          <t>$1,200-$11,000/mo</t>
+        </is>
+      </c>
+      <c r="E21" s="7" t="inlineStr">
+        <is>
+          <t>Capitol Outdoor</t>
+        </is>
+      </c>
+      <c r="F21" s="7" t="inlineStr">
+        <is>
+          <t>KXTV 10 · KOVR 13 · KCRA 3 · KTXL Fox 40</t>
+        </is>
+      </c>
+      <c r="G21" s="7" t="inlineStr">
+        <is>
+          <t>iHeart (KFBK) · Audacy · Bonneville</t>
+        </is>
+      </c>
+      <c r="H21" s="7" t="inlineStr">
+        <is>
+          <t>The Sacramento Bee</t>
+        </is>
+      </c>
+      <c r="I21" s="7" t="inlineStr">
+        <is>
+          <t>The Glass Agency, Position Interactive</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="B22" s="7" t="inlineStr">
+        <is>
+          <t>Orlando</t>
+        </is>
+      </c>
+      <c r="C22" s="6" t="inlineStr">
+        <is>
+          <t>2.8M</t>
+        </is>
+      </c>
+      <c r="D22" s="6" t="inlineStr">
+        <is>
+          <t>$1,200-$12,000/mo</t>
+        </is>
+      </c>
+      <c r="E22" s="7" t="inlineStr">
+        <is>
+          <t>Orlando Outdoor</t>
+        </is>
+      </c>
+      <c r="F22" s="7" t="inlineStr">
+        <is>
+          <t>WFTV 9 · WKMG 6 · WESH 2 · WOFL Fox 35</t>
+        </is>
+      </c>
+      <c r="G22" s="7" t="inlineStr">
+        <is>
+          <t>iHeart · Cox (WDBO)</t>
+        </is>
+      </c>
+      <c r="H22" s="7" t="inlineStr">
+        <is>
+          <t>Orlando Sentinel</t>
+        </is>
+      </c>
+      <c r="I22" s="7" t="inlineStr">
+        <is>
+          <t>&amp;Barr, PUSH</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="6" t="n">
+        <v>21</v>
+      </c>
+      <c r="B23" s="7" t="inlineStr">
+        <is>
+          <t>St. Louis</t>
+        </is>
+      </c>
+      <c r="C23" s="6" t="inlineStr">
+        <is>
+          <t>2.8M</t>
+        </is>
+      </c>
+      <c r="D23" s="6" t="inlineStr">
+        <is>
+          <t>$1,000-$10,000/mo</t>
+        </is>
+      </c>
+      <c r="E23" s="7" t="inlineStr">
+        <is>
+          <t>DDI Media, Robinson Outdoor</t>
+        </is>
+      </c>
+      <c r="F23" s="7" t="inlineStr">
+        <is>
+          <t>KDNL 30 · KMOV 4 · KSDK 5 · KTVI Fox 2</t>
+        </is>
+      </c>
+      <c r="G23" s="7" t="inlineStr">
+        <is>
+          <t>Audacy (KMOX) · iHeart · Hubbard</t>
+        </is>
+      </c>
+      <c r="H23" s="7" t="inlineStr">
+        <is>
+          <t>St. Louis Post-Dispatch</t>
+        </is>
+      </c>
+      <c r="I23" s="7" t="inlineStr">
+        <is>
+          <t>HLK, Rodgers Townsend (DDB)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="6" t="n">
+        <v>22</v>
+      </c>
+      <c r="B24" s="7" t="inlineStr">
+        <is>
+          <t>Pittsburgh</t>
+        </is>
+      </c>
+      <c r="C24" s="6" t="inlineStr">
+        <is>
+          <t>2.4M</t>
+        </is>
+      </c>
+      <c r="D24" s="6" t="inlineStr">
+        <is>
+          <t>$1,000-$9,000/mo</t>
+        </is>
+      </c>
+      <c r="E24" s="7" t="inlineStr">
+        <is>
+          <t>Penneco Outdoor Advertising, Steel City Billboards, TM Advertising</t>
+        </is>
+      </c>
+      <c r="F24" s="7" t="inlineStr">
+        <is>
+          <t>WTAE 4 · KDKA 2 · WPXI 11 · WPGH Fox 53</t>
+        </is>
+      </c>
+      <c r="G24" s="7" t="inlineStr">
+        <is>
+          <t>Audacy (KDKA) · iHeart (WDVE) · Steel City Media</t>
+        </is>
+      </c>
+      <c r="H24" s="7" t="inlineStr">
+        <is>
+          <t>Pittsburgh Post-Gazette</t>
+        </is>
+      </c>
+      <c r="I24" s="7" t="inlineStr">
+        <is>
+          <t>Brunner, MARC USA (legacy), Gatesman</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="6" t="n">
+        <v>23</v>
+      </c>
+      <c r="B25" s="7" t="inlineStr">
+        <is>
+          <t>San Diego</t>
+        </is>
+      </c>
+      <c r="C25" s="6" t="inlineStr">
+        <is>
+          <t>3.3M</t>
+        </is>
+      </c>
+      <c r="D25" s="6" t="inlineStr">
+        <is>
+          <t>$1,500-$10,000/mo</t>
+        </is>
+      </c>
+      <c r="E25" s="7" t="inlineStr">
+        <is>
+          <t>American Outdoor Advertising, Capitol Outdoor, Bray Outdoor Ads</t>
+        </is>
+      </c>
+      <c r="F25" s="7" t="inlineStr">
+        <is>
+          <t>KGTV 10 · KFMB 8 · KNSD 7/39 · KSWB Fox 5</t>
+        </is>
+      </c>
+      <c r="G25" s="7" t="inlineStr">
+        <is>
+          <t>iHeart (KOGO) · Audacy · Local Media San Diego</t>
+        </is>
+      </c>
+      <c r="H25" s="7" t="inlineStr">
+        <is>
+          <t>The San Diego Union-Tribune</t>
+        </is>
+      </c>
+      <c r="I25" s="7" t="inlineStr">
+        <is>
+          <t>VITRO (Petco work), i.d.e.a.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="6" t="n">
+        <v>24</v>
+      </c>
+      <c r="B26" s="7" t="inlineStr">
+        <is>
+          <t>Baltimore</t>
+        </is>
+      </c>
+      <c r="C26" s="6" t="inlineStr">
+        <is>
+          <t>2.8M</t>
+        </is>
+      </c>
+      <c r="D26" s="6" t="inlineStr">
+        <is>
+          <t>$1,200-$11,000/mo</t>
+        </is>
+      </c>
+      <c r="E26" s="7" t="inlineStr">
+        <is>
+          <t>Vision Outdoor</t>
+        </is>
+      </c>
+      <c r="F26" s="7" t="inlineStr">
+        <is>
+          <t>WMAR 2 · WJZ 13 · WBAL 11 · WBFF Fox 45</t>
+        </is>
+      </c>
+      <c r="G26" s="7" t="inlineStr">
+        <is>
+          <t>Hearst (WBAL radio) · iHeart · Audacy</t>
+        </is>
+      </c>
+      <c r="H26" s="7" t="inlineStr">
+        <is>
+          <t>The Baltimore Sun</t>
+        </is>
+      </c>
+      <c r="I26" s="7" t="inlineStr">
+        <is>
+          <t>Planit, GKV, idfive</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="6" t="n">
+        <v>25</v>
+      </c>
+      <c r="B27" s="7" t="inlineStr">
+        <is>
+          <t>Charlotte</t>
+        </is>
+      </c>
+      <c r="C27" s="6" t="inlineStr">
+        <is>
+          <t>2.8M</t>
+        </is>
+      </c>
+      <c r="D27" s="6" t="inlineStr">
+        <is>
+          <t>$1,000-$9,000/mo</t>
+        </is>
+      </c>
+      <c r="E27" s="7" t="inlineStr">
+        <is>
+          <t>Allison Outdoor Advertising, Adams Outdoor Advertising, Trailhead Media</t>
+        </is>
+      </c>
+      <c r="F27" s="7" t="inlineStr">
+        <is>
+          <t>WSOC 9 · WBTV 3 · WCNC 36 · WJZY Fox 46</t>
+        </is>
+      </c>
+      <c r="G27" s="7" t="inlineStr">
+        <is>
+          <t>iHeart · Urban One · Norsan Media (Spanish, local)</t>
+        </is>
+      </c>
+      <c r="H27" s="7" t="inlineStr">
+        <is>
+          <t>The Charlotte Observer</t>
+        </is>
+      </c>
+      <c r="I27" s="7" t="inlineStr">
+        <is>
+          <t>Wray Ward, Luquire</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="6" t="n">
+        <v>26</v>
+      </c>
+      <c r="B28" s="7" t="inlineStr">
+        <is>
+          <t>Raleigh</t>
+        </is>
+      </c>
+      <c r="C28" s="6" t="inlineStr">
+        <is>
+          <t>1.5M (Triangle ~2.1M)</t>
+        </is>
+      </c>
+      <c r="D28" s="6" t="inlineStr">
+        <is>
+          <t>$1,000-$10,000/mo</t>
+        </is>
+      </c>
+      <c r="E28" s="7" t="inlineStr">
+        <is>
+          <t>Allison Outdoor Advertising, Adams Outdoor Advertising, Trailhead Media</t>
+        </is>
+      </c>
+      <c r="F28" s="7" t="inlineStr">
+        <is>
+          <t>WTVD 11 · WNCN 17 · WRAL 5 · WRAZ Fox 50</t>
+        </is>
+      </c>
+      <c r="G28" s="7" t="inlineStr">
+        <is>
+          <t>iHeart · Curtis Media (local Triangle) · Capitol Broadcasting</t>
+        </is>
+      </c>
+      <c r="H28" s="7" t="inlineStr">
+        <is>
+          <t>The News &amp; Observer</t>
+        </is>
+      </c>
+      <c r="I28" s="7" t="inlineStr">
+        <is>
+          <t>McKinney (Durham), Baldwin&amp;</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="6" t="n">
+        <v>27</v>
+      </c>
+      <c r="B29" s="7" t="inlineStr">
+        <is>
+          <t>Indianapolis</t>
+        </is>
+      </c>
+      <c r="C29" s="6" t="inlineStr">
+        <is>
+          <t>2.1M</t>
+        </is>
+      </c>
+      <c r="D29" s="6" t="inlineStr">
+        <is>
+          <t>$1,000-$10,000/mo</t>
+        </is>
+      </c>
+      <c r="E29" s="7" t="inlineStr">
+        <is>
+          <t>Reagan Outdoor Advertising, Keyes Outdoor Advertising</t>
+        </is>
+      </c>
+      <c r="F29" s="7" t="inlineStr">
+        <is>
+          <t>WRTV 6 · WTTV 4 · WTHR 13 · WXIN Fox 59</t>
+        </is>
+      </c>
+      <c r="G29" s="7" t="inlineStr">
+        <is>
+          <t>iHeart · Cumulus (WFMS) · Urban One</t>
+        </is>
+      </c>
+      <c r="H29" s="7" t="inlineStr">
+        <is>
+          <t>The Indianapolis Star</t>
+        </is>
+      </c>
+      <c r="I29" s="7" t="inlineStr">
+        <is>
+          <t>Young &amp; Laramore, Hirons</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="6" t="n">
+        <v>28</v>
+      </c>
+      <c r="B30" s="7" t="inlineStr">
+        <is>
+          <t>Cincinnati</t>
+        </is>
+      </c>
+      <c r="C30" s="6" t="inlineStr">
+        <is>
+          <t>2.3M</t>
+        </is>
+      </c>
+      <c r="D30" s="6" t="inlineStr">
+        <is>
+          <t>$1,000-$10,000/mo</t>
+        </is>
+      </c>
+      <c r="E30" s="7" t="inlineStr">
+        <is>
+          <t>American Outdoor Advertising (Columbus), Outdoor Advertising Center, Key-Ads, Inc.</t>
+        </is>
+      </c>
+      <c r="F30" s="7" t="inlineStr">
+        <is>
+          <t>WCPO 9 · WKRC 12 · WLWT 5 · WXIX Fox 19</t>
+        </is>
+      </c>
+      <c r="G30" s="7" t="inlineStr">
+        <is>
+          <t>iHeart (700WLW) · Hubbard (WKRQ) · Cumulus</t>
+        </is>
+      </c>
+      <c r="H30" s="7" t="inlineStr">
+        <is>
+          <t>The Cincinnati Enquirer</t>
+        </is>
+      </c>
+      <c r="I30" s="7" t="inlineStr">
+        <is>
+          <t>Curiosity, Barefoot Proximity (BBDO)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="6" t="n">
+        <v>29</v>
+      </c>
+      <c r="B31" s="7" t="inlineStr">
+        <is>
+          <t>Las Vegas</t>
+        </is>
+      </c>
+      <c r="C31" s="6" t="inlineStr">
+        <is>
+          <t>2.3M</t>
+        </is>
+      </c>
+      <c r="D31" s="6" t="inlineStr">
+        <is>
+          <t>$1,500-$25,000/mo</t>
+        </is>
+      </c>
+      <c r="E31" s="7" t="inlineStr">
+        <is>
+          <t>Reagan Outdoor Advertising, Las Vegas Billboards</t>
+        </is>
+      </c>
+      <c r="F31" s="7" t="inlineStr">
+        <is>
+          <t>KTNV 13 · KLAS 8 · KSNV 3 · KVVU Fox 5</t>
+        </is>
+      </c>
+      <c r="G31" s="7" t="inlineStr">
+        <is>
+          <t>Audacy · iHeart · Lotus (local)</t>
+        </is>
+      </c>
+      <c r="H31" s="7" t="inlineStr">
+        <is>
+          <t>Las Vegas Review-Journal</t>
+        </is>
+      </c>
+      <c r="I31" s="7" t="inlineStr">
+        <is>
+          <t>R&amp;R Partners ('What happens here, stays here')</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="6" t="n">
+        <v>30</v>
+      </c>
+      <c r="B32" s="7" t="inlineStr">
+        <is>
+          <t>San Antonio</t>
+        </is>
+      </c>
+      <c r="C32" s="6" t="inlineStr">
+        <is>
+          <t>2.6M</t>
+        </is>
+      </c>
+      <c r="D32" s="6" t="inlineStr">
+        <is>
+          <t>$1,000-$8,000/mo</t>
+        </is>
+      </c>
+      <c r="E32" s="7" t="inlineStr">
+        <is>
+          <t>SignAd Outdoor Advertising, Gilbreath Outdoor Advertising, Lux Media</t>
+        </is>
+      </c>
+      <c r="F32" s="7" t="inlineStr">
+        <is>
+          <t>KSAT 12 · KENS 5 · WOAI 4 · KABB Fox 29</t>
+        </is>
+      </c>
+      <c r="G32" s="7" t="inlineStr">
+        <is>
+          <t>iHeartMedia (corporate HQ — WOAI) · Cox · Univision (Spanish)</t>
+        </is>
+      </c>
+      <c r="H32" s="7" t="inlineStr">
+        <is>
+          <t>San Antonio Express-News</t>
+        </is>
+      </c>
+      <c r="I32" s="7" t="inlineStr">
+        <is>
+          <t>The Atkins Group, Giles-Parscale (legacy)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="6" t="n">
+        <v>31</v>
+      </c>
+      <c r="B33" s="7" t="inlineStr">
+        <is>
+          <t>Portland</t>
+        </is>
+      </c>
+      <c r="C33" s="6" t="inlineStr">
+        <is>
+          <t>2.5M</t>
+        </is>
+      </c>
+      <c r="D33" s="6" t="inlineStr">
+        <is>
+          <t>$1,200-$11,000/mo</t>
+        </is>
+      </c>
+      <c r="E33" s="7" t="inlineStr">
+        <is>
+          <t>Grapevine Outdoor, New Tradition Media, Meadow Outdoor Advertising</t>
+        </is>
+      </c>
+      <c r="F33" s="7" t="inlineStr">
+        <is>
+          <t>KATU 2 · KOIN 6 · KGW 8 · KPTV Fox 12</t>
+        </is>
+      </c>
+      <c r="G33" s="7" t="inlineStr">
+        <is>
+          <t>iHeart (KEX) · Audacy · Alpha Media (HQ Portland)</t>
+        </is>
+      </c>
+      <c r="H33" s="7" t="inlineStr">
+        <is>
+          <t>The Oregonian</t>
+        </is>
+      </c>
+      <c r="I33" s="7" t="inlineStr">
+        <is>
+          <t>Wieden+Kennedy (HQ), Instrument, Opinionated</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="6" t="n">
+        <v>32</v>
+      </c>
+      <c r="B34" s="7" t="inlineStr">
+        <is>
+          <t>Milwaukee</t>
+        </is>
+      </c>
+      <c r="C34" s="6" t="inlineStr">
+        <is>
+          <t>1.6M</t>
+        </is>
+      </c>
+      <c r="D34" s="6" t="inlineStr">
+        <is>
+          <t>$1,000-$10,000/mo</t>
+        </is>
+      </c>
+      <c r="E34" s="7" t="inlineStr">
+        <is>
+          <t>Outdoor Advertising Center</t>
+        </is>
+      </c>
+      <c r="F34" s="7" t="inlineStr">
+        <is>
+          <t>WISN 12 · WDJT 58 · WTMJ 4 · WITI Fox 6</t>
+        </is>
+      </c>
+      <c r="G34" s="7" t="inlineStr">
+        <is>
+          <t>Good Karma (WTMJ radio) · iHeart · Saga (WKLH)</t>
+        </is>
+      </c>
+      <c r="H34" s="7" t="inlineStr">
+        <is>
+          <t>Milwaukee Journal Sentinel</t>
+        </is>
+      </c>
+      <c r="I34" s="7" t="inlineStr">
+        <is>
+          <t>Cramer-Krasselt, BVK, Hoffman York</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="6" t="n">
+        <v>33</v>
+      </c>
+      <c r="B35" s="7" t="inlineStr">
+        <is>
+          <t>Columbus</t>
+        </is>
+      </c>
+      <c r="C35" s="6" t="inlineStr">
+        <is>
+          <t>2.2M</t>
+        </is>
+      </c>
+      <c r="D35" s="6" t="inlineStr">
+        <is>
+          <t>$1,000-$9,000/mo</t>
+        </is>
+      </c>
+      <c r="E35" s="7" t="inlineStr">
+        <is>
+          <t>American Outdoor Advertising (Columbus), Outdoor Advertising Center, Kenjoh Outdoor</t>
+        </is>
+      </c>
+      <c r="F35" s="7" t="inlineStr">
+        <is>
+          <t>WSYX 6 · WBNS 10 · WCMH 4 · WTTE Fox 28</t>
+        </is>
+      </c>
+      <c r="G35" s="7" t="inlineStr">
+        <is>
+          <t>iHeart (WTVN/WNCI) · Saga (WSNY) · Urban One</t>
+        </is>
+      </c>
+      <c r="H35" s="7" t="inlineStr">
+        <is>
+          <t>The Columbus Dispatch</t>
+        </is>
+      </c>
+      <c r="I35" s="7" t="inlineStr">
+        <is>
+          <t>Fahlgren Mortine, The Shipyard, Ologie</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="6" t="n">
+        <v>34</v>
+      </c>
+      <c r="B36" s="7" t="inlineStr">
+        <is>
+          <t>Kansas City</t>
+        </is>
+      </c>
+      <c r="C36" s="6" t="inlineStr">
+        <is>
+          <t>2.2M</t>
+        </is>
+      </c>
+      <c r="D36" s="6" t="inlineStr">
+        <is>
+          <t>$1,000-$9,000/mo</t>
+        </is>
+      </c>
+      <c r="E36" s="7" t="inlineStr">
+        <is>
+          <t>Ad-Trend, Midwest Billboards</t>
+        </is>
+      </c>
+      <c r="F36" s="7" t="inlineStr">
+        <is>
+          <t>KMBC 9 · KCTV 5 · KSHB 41 · WDAF Fox 4</t>
+        </is>
+      </c>
+      <c r="G36" s="7" t="inlineStr">
+        <is>
+          <t>Audacy (KMBZ) · Cumulus · Carter Broadcast (KPRS)</t>
+        </is>
+      </c>
+      <c r="H36" s="7" t="inlineStr">
+        <is>
+          <t>The Kansas City Star</t>
+        </is>
+      </c>
+      <c r="I36" s="7" t="inlineStr">
+        <is>
+          <t>VML (HQ), Barkley OKRP</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="6" t="n">
+        <v>35</v>
+      </c>
+      <c r="B37" s="7" t="inlineStr">
+        <is>
+          <t>Nashville</t>
+        </is>
+      </c>
+      <c r="C37" s="6" t="inlineStr">
+        <is>
+          <t>2.1M</t>
+        </is>
+      </c>
+      <c r="D37" s="6" t="inlineStr">
+        <is>
+          <t>$1,200-$11,000/mo</t>
+        </is>
+      </c>
+      <c r="E37" s="7" t="inlineStr">
+        <is>
+          <t>Allison Outdoor Advertising</t>
+        </is>
+      </c>
+      <c r="F37" s="7" t="inlineStr">
+        <is>
+          <t>WKRN 2 · WTVF 5 · WSMV 4 · WZTV Fox 17</t>
+        </is>
+      </c>
+      <c r="G37" s="7" t="inlineStr">
+        <is>
+          <t>iHeart (WLAC) · Cumulus (WKDF/WSM-FM) · Opry Ent. (WSM-AM)</t>
+        </is>
+      </c>
+      <c r="H37" s="7" t="inlineStr">
+        <is>
+          <t>The Tennessean</t>
+        </is>
+      </c>
+      <c r="I37" s="7" t="inlineStr">
+        <is>
+          <t>bohan, GS&amp;F</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="6" t="n">
+        <v>36</v>
+      </c>
+      <c r="B38" s="7" t="inlineStr">
+        <is>
+          <t>Salt Lake City</t>
+        </is>
+      </c>
+      <c r="C38" s="6" t="inlineStr">
+        <is>
+          <t>1.3M</t>
+        </is>
+      </c>
+      <c r="D38" s="6" t="inlineStr">
+        <is>
+          <t>$1,000-$9,000/mo</t>
+        </is>
+      </c>
+      <c r="E38" s="7" t="inlineStr">
+        <is>
+          <t>Reagan Outdoor Advertising, YESCO Outdoor Media</t>
+        </is>
+      </c>
+      <c r="F38" s="7" t="inlineStr">
+        <is>
+          <t>KTVX 4 · KUTV 2 · KSL 5 · KSTU Fox 13</t>
+        </is>
+      </c>
+      <c r="G38" s="7" t="inlineStr">
+        <is>
+          <t>Bonneville (HQ — KSL) · iHeart · Broadway Media (local)</t>
+        </is>
+      </c>
+      <c r="H38" s="7" t="inlineStr">
+        <is>
+          <t>The Salt Lake Tribune / Deseret News</t>
+        </is>
+      </c>
+      <c r="I38" s="7" t="inlineStr">
+        <is>
+          <t>Struck, Love Communications, Richter7</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="6" t="n">
+        <v>37</v>
+      </c>
+      <c r="B39" s="7" t="inlineStr">
+        <is>
+          <t>New Orleans</t>
+        </is>
+      </c>
+      <c r="C39" s="6" t="inlineStr">
+        <is>
+          <t>1.3M</t>
+        </is>
+      </c>
+      <c r="D39" s="6" t="inlineStr">
+        <is>
+          <t>$1,000-$11,000/mo</t>
+        </is>
+      </c>
+      <c r="E39" s="7" t="inlineStr">
+        <is>
+          <t>Lindmark Outdoor Media</t>
+        </is>
+      </c>
+      <c r="F39" s="7" t="inlineStr">
+        <is>
+          <t>WGNO 26 · WWL 4 · WDSU 6 · WVUE Fox 8</t>
+        </is>
+      </c>
+      <c r="G39" s="7" t="inlineStr">
+        <is>
+          <t>Audacy (WWL radio) · iHeart · Cumulus</t>
+        </is>
+      </c>
+      <c r="H39" s="7" t="inlineStr">
+        <is>
+          <t>The Times-Picayune / NOLA.com / The Advocate</t>
+        </is>
+      </c>
+      <c r="I39" s="7" t="inlineStr">
+        <is>
+          <t>Peter Mayer, Trumpet</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="6" t="n">
+        <v>38</v>
+      </c>
+      <c r="B40" s="7" t="inlineStr">
+        <is>
+          <t>Oklahoma City</t>
+        </is>
+      </c>
+      <c r="C40" s="6" t="inlineStr">
+        <is>
+          <t>1.5M</t>
+        </is>
+      </c>
+      <c r="D40" s="6" t="inlineStr">
+        <is>
+          <t>$900-$8,000/mo</t>
+        </is>
+      </c>
+      <c r="E40" s="7" t="inlineStr">
+        <is>
+          <t>Headrick Outdoor Media, Lindmark Outdoor Media</t>
+        </is>
+      </c>
+      <c r="F40" s="7" t="inlineStr">
+        <is>
+          <t>KOCO 5 · KWTV 9 · KFOR 4 · KOKH Fox 25</t>
+        </is>
+      </c>
+      <c r="G40" s="7" t="inlineStr">
+        <is>
+          <t>iHeart (KTOK) · Cumulus (KATT) · Tyler Media (local)</t>
+        </is>
+      </c>
+      <c r="H40" s="7" t="inlineStr">
+        <is>
+          <t>The Oklahoman</t>
+        </is>
+      </c>
+      <c r="I40" s="7" t="inlineStr">
+        <is>
+          <t>Ackerman McQueen, VI Marketing + Branding</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="6" t="n">
+        <v>39</v>
+      </c>
+      <c r="B41" s="7" t="inlineStr">
+        <is>
+          <t>Memphis</t>
+        </is>
+      </c>
+      <c r="C41" s="6" t="inlineStr">
+        <is>
+          <t>1.3M</t>
+        </is>
+      </c>
+      <c r="D41" s="6" t="inlineStr">
+        <is>
+          <t>$900-$8,000/mo</t>
+        </is>
+      </c>
+      <c r="E41" s="7" t="inlineStr">
+        <is>
+          <t>Allison Outdoor Advertising</t>
+        </is>
+      </c>
+      <c r="F41" s="7" t="inlineStr">
+        <is>
+          <t>WATN 24 · WREG 3 · WMC 5 · WHBQ Fox 13</t>
+        </is>
+      </c>
+      <c r="G41" s="7" t="inlineStr">
+        <is>
+          <t>iHeart · Cumulus · Flinn Broadcasting (local)</t>
+        </is>
+      </c>
+      <c r="H41" s="7" t="inlineStr">
+        <is>
+          <t>The Commercial Appeal</t>
+        </is>
+      </c>
+      <c r="I41" s="7" t="inlineStr">
+        <is>
+          <t>archer malmo (Signet), Sullivan Branding</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="6" t="n">
+        <v>40</v>
+      </c>
+      <c r="B42" s="7" t="inlineStr">
+        <is>
+          <t>Richmond</t>
+        </is>
+      </c>
+      <c r="C42" s="6" t="inlineStr">
+        <is>
+          <t>1.3M</t>
+        </is>
+      </c>
+      <c r="D42" s="6" t="inlineStr">
+        <is>
+          <t>$900-$8,000/mo</t>
+        </is>
+      </c>
+      <c r="E42" s="7" t="inlineStr">
+        <is>
+          <t>Lamar / Clear Channel / OUTFRONT</t>
+        </is>
+      </c>
+      <c r="F42" s="7" t="inlineStr">
+        <is>
+          <t>WRIC 8 · WTVR 6 · WWBT 12 · WRLH Fox 35</t>
+        </is>
+      </c>
+      <c r="G42" s="7" t="inlineStr">
+        <is>
+          <t>Audacy (WRVA) · SummitMedia · Urban One</t>
+        </is>
+      </c>
+      <c r="H42" s="7" t="inlineStr">
+        <is>
+          <t>Richmond Times-Dispatch</t>
+        </is>
+      </c>
+      <c r="I42" s="7" t="inlineStr">
+        <is>
+          <t>The Martin Agency (GEICO), Arts &amp; Letters</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="6" t="n">
+        <v>41</v>
+      </c>
+      <c r="B43" s="7" t="inlineStr">
+        <is>
+          <t>Austin</t>
+        </is>
+      </c>
+      <c r="C43" s="6" t="inlineStr">
+        <is>
+          <t>2.5M</t>
+        </is>
+      </c>
+      <c r="D43" s="6" t="inlineStr">
+        <is>
+          <t>$1,200-$12,000/mo</t>
+        </is>
+      </c>
+      <c r="E43" s="7" t="inlineStr">
+        <is>
+          <t>Reagan Outdoor Advertising, Lux Media, Burkett Media</t>
+        </is>
+      </c>
+      <c r="F43" s="7" t="inlineStr">
+        <is>
+          <t>KVUE 24 · KEYE 42 · KXAN 36 · KTBC Fox 7</t>
+        </is>
+      </c>
+      <c r="G43" s="7" t="inlineStr">
+        <is>
+          <t>iHeart · Audacy · Waterloo Media (local — KLBJ)</t>
+        </is>
+      </c>
+      <c r="H43" s="7" t="inlineStr">
+        <is>
+          <t>Austin American-Statesman</t>
+        </is>
+      </c>
+      <c r="I43" s="7" t="inlineStr">
+        <is>
+          <t>GSD&amp;M (HQ), McGarrah Jessee, Preacher</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="6" t="n">
+        <v>42</v>
+      </c>
+      <c r="B44" s="7" t="inlineStr">
+        <is>
+          <t>Jacksonville</t>
+        </is>
+      </c>
+      <c r="C44" s="6" t="inlineStr">
+        <is>
+          <t>1.7M</t>
+        </is>
+      </c>
+      <c r="D44" s="6" t="inlineStr">
+        <is>
+          <t>$800-$6,000/mo</t>
+        </is>
+      </c>
+      <c r="E44" s="7" t="inlineStr">
+        <is>
+          <t>Digital Outdoor Advertising, LLC, American Mobile Ads, Daily Billboards</t>
+        </is>
+      </c>
+      <c r="F44" s="7" t="inlineStr">
+        <is>
+          <t>WJXX 25 · WJAX 47 · WTLV 12 · WFOX 30</t>
+        </is>
+      </c>
+      <c r="G44" s="7" t="inlineStr">
+        <is>
+          <t>Cox (WOKV/WAPE) · iHeart</t>
+        </is>
+      </c>
+      <c r="H44" s="7" t="inlineStr">
+        <is>
+          <t>The Florida Times-Union</t>
+        </is>
+      </c>
+      <c r="I44" s="7" t="inlineStr">
+        <is>
+          <t>Dalton Agency, Shepherd (St. John &amp; Partners)</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="30" customHeight="1">
+      <c r="A46" s="11" t="inlineStr">
+        <is>
+          <t>UNIVERSAL FOUNDATION (every metro, before any media buy): 1) Google Business Profile + Local Services Ads + review engine  2) City landing pages + local SEO  3) Geofenced social + search ads + retargeting  4) Then buy local media below.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A2:I44"/>
+  <mergeCells count="2">
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A46:I46"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:D20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>

</xml_diff>